<commit_message>
feat: add public booking and room calendar
</commit_message>
<xml_diff>
--- a/docs/仕様書/民宿管理システム.xlsx
+++ b/docs/仕様書/民宿管理システム.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表紙" sheetId="1" r:id="R9cd7b69ccb6f4e99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="変更履歴" sheetId="2" r:id="Re74d94373cfb43c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概要" sheetId="3" r:id="R3eaf500c5a65411e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="業務要件" sheetId="4" r:id="Ra831eb4fc98c4bfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="機能一覧" sheetId="5" r:id="R6aedfd71e5eb4abd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="コード行別処理仕様" sheetId="6" r:id="R507e02ee0b114440"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="画面一覧" sheetId="7" r:id="Ra104d3174bab4076"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB設計" sheetId="8" r:id="R4bbbaa26f9dc4454"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API一覧" sheetId="9" r:id="Rc0e5e19070b14562"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非機能要件" sheetId="10" r:id="R0a6c50e9b8d547bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="テスト仕様" sheetId="11" r:id="R41a3aac06fba4453"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="スケジュール" sheetId="12" r:id="R496578be69704415"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参考資料" sheetId="13" r:id="Re4683b0b383f46bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="運用・基盤仕様" sheetId="14" r:id="R6a1788ca72424301"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表紙" sheetId="1" r:id="R7b225ec44a0f4fb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="変更履歴" sheetId="2" r:id="R42d10e4788c24613"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概要" sheetId="3" r:id="R744e4b4813664c0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="業務要件" sheetId="4" r:id="R1dc6210e5c2c482d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="機能一覧" sheetId="5" r:id="Rd2d1ad6afb2a47ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="コード行別処理仕様" sheetId="6" r:id="Rf864c2e9212240fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="画面一覧" sheetId="7" r:id="R9ccce087721b4202"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB設計" sheetId="8" r:id="R07cf62bf5e594390"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API一覧" sheetId="9" r:id="R0cf49fd4a759426a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非機能要件" sheetId="10" r:id="Ref6a70ff613f4abd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="テスト仕様" sheetId="11" r:id="R41fa0e7b42db43d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="スケジュール" sheetId="12" r:id="R97cda7e3cce3402e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参考資料" sheetId="13" r:id="R297e11a80baa4971"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="運用・基盤仕様" sheetId="14" r:id="R9db09c5e379f4a58"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -176,7 +176,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="40">
+  <x:cellXfs count="42">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -294,6 +294,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -558,7 +564,7 @@
         <x:v>何念童</x:v>
       </x:c>
       <x:c r="C3" s="27" t="str">
-        <x:v>2026-07-13</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="D3" s="27" t="str">
         <x:v>何念童</x:v>
@@ -570,7 +576,7 @@
         <x:v>備考</x:v>
       </x:c>
       <x:c r="B4" s="27" t="str">
-        <x:v>現行 Spring Boot + React + MyBatis 実装を基準に更新</x:v>
+        <x:v>現行 Spring Boot + React + MyBatis 実装と管理端房態カレンダー v1.11 を基準に更新</x:v>
       </x:c>
       <x:c r="C4" s="26" t="str">
         <x:v>対象シート</x:v>
@@ -668,7 +674,7 @@
         <x:v>版数</x:v>
       </x:c>
       <x:c r="B12" s="30" t="str">
-        <x:v>1.9</x:v>
+        <x:v>1.11</x:v>
       </x:c>
       <x:c r="C12" s="30"/>
       <x:c r="D12" s="29" t="str">
@@ -683,7 +689,7 @@
         <x:v>更新日</x:v>
       </x:c>
       <x:c r="B13" s="30" t="str">
-        <x:v>2026-07-13</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="C13" s="30"/>
       <x:c r="D13" s="29" t="str">
@@ -965,7 +971,7 @@
         <x:v>何念童</x:v>
       </x:c>
       <x:c r="C3" s="27" t="str">
-        <x:v>2026-07-13</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="D3" s="27" t="str">
         <x:v>何念童</x:v>
@@ -1322,6 +1328,57 @@
       </x:c>
       <x:c r="E25" s="19" t="str">
         <x:v>公開URLと拒否URLが明示されていること。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="36" customHeight="1">
+      <x:c r="A26" s="40" t="str">
+        <x:v>CAL-NF-001</x:v>
+      </x:c>
+      <x:c r="B26" s="40" t="str">
+        <x:v>整合性</x:v>
+      </x:c>
+      <x:c r="C26" s="40" t="str">
+        <x:v>二重予約・二重ブロック防止</x:v>
+      </x:c>
+      <x:c r="D26" s="40" t="str">
+        <x:v>ServiceロックとPostgreSQL排他制約／triggerで競合を拒否する。</x:v>
+      </x:c>
+      <x:c r="E26" s="40" t="str">
+        <x:v>高</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="36" customHeight="1">
+      <x:c r="A27" s="40" t="str">
+        <x:v>CAL-NF-002</x:v>
+      </x:c>
+      <x:c r="B27" s="40" t="str">
+        <x:v>更新</x:v>
+      </x:c>
+      <x:c r="C27" s="40" t="str">
+        <x:v>最新状態反映</x:v>
+      </x:c>
+      <x:c r="D27" s="40" t="str">
+        <x:v>表示中のみ30秒間隔で再取得し、復帰時にも更新する。</x:v>
+      </x:c>
+      <x:c r="E27" s="40" t="str">
+        <x:v>高</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="36" customHeight="1">
+      <x:c r="A28" s="40" t="str">
+        <x:v>CAL-NF-003</x:v>
+      </x:c>
+      <x:c r="B28" s="40" t="str">
+        <x:v>監査</x:v>
+      </x:c>
+      <x:c r="C28" s="40" t="str">
+        <x:v>在庫変更履歴</x:v>
+      </x:c>
+      <x:c r="D28" s="40" t="str">
+        <x:v>ブロック変更はbefore/after、操作者、時刻を追記保存する。</x:v>
+      </x:c>
+      <x:c r="E28" s="40" t="str">
+        <x:v>高</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1395,7 +1452,7 @@
         <x:v>何念童</x:v>
       </x:c>
       <x:c r="C3" s="27" t="str">
-        <x:v>2026-07-13</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="D3" s="27" t="str">
         <x:v>何念童</x:v>
@@ -1707,7 +1764,7 @@
         <x:v>全 JUnit5 テスト / TestResultLogger</x:v>
       </x:c>
       <x:c r="F14" s="30" t="str">
-        <x:v>106件のテストが同じ証跡形式で実行され、全件成功する。</x:v>
+        <x:v>123件のテストが同じ証跡形式で実行され、全件成功する。</x:v>
       </x:c>
       <x:c r="G14" s="30" t="str">
         <x:v>中</x:v>
@@ -1720,7 +1777,7 @@
       </x:c>
       <x:c r="J14" s="30"/>
       <x:c r="K14" s="30" t="str">
-        <x:v>2026-07-13 mvn test: 106件成功</x:v>
+        <x:v>2026-09-02 mvn verify: 123件成功</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -2943,13 +3000,13 @@
         <x:v>@LoggedTest と TestResultLogger が全テストクラスに適用されている。</x:v>
       </x:c>
       <x:c r="F50" s="30" t="str">
-        <x:v>mvn test を実行</x:v>
+        <x:v>123件すべてで test_XX、注解、文字列結果を出力し成功する。</x:v>
       </x:c>
       <x:c r="G50" s="30" t="str">
         <x:v>106件すべてで test_XX、注解、文字列結果を出力し成功する。</x:v>
       </x:c>
       <x:c r="H50" s="30" t="str">
-        <x:v>Surefire: Tests run 106 / Failures 0 / Errors 0 / Skipped 0</x:v>
+        <x:v>Surefire: Tests run 123 / Failures 0 / Errors 0 / Skipped 0</x:v>
       </x:c>
       <x:c r="I50" s="30" t="str">
         <x:v>TREQ-008</x:v>
@@ -3236,6 +3293,227 @@
         <x:v>CI改善候補</x:v>
       </x:c>
       <x:c r="K58" s="19"/>
+    </x:row>
+    <x:row r="59" ht="15" hidden="0" customHeight="1">
+      <x:c r="A59" t="str">
+        <x:v>UT-043</x:v>
+      </x:c>
+      <x:c r="B59" t="str">
+        <x:v>ReservationService.findAvailableRooms</x:v>
+      </x:c>
+      <x:c r="C59" t="str">
+        <x:v>日程・人数に合う客室だけを提示したい。</x:v>
+      </x:c>
+      <x:c r="D59" t="str">
+        <x:v>期間重複、定員、当日房態をまとめて判定すること。</x:v>
+      </x:c>
+      <x:c r="E59" t="str">
+        <x:v>複数客室と既存予約あり</x:v>
+      </x:c>
+      <x:c r="F59" t="str">
+        <x:v>日程・人数を指定</x:v>
+      </x:c>
+      <x:c r="G59" t="str">
+        <x:v>条件一致する客室だけ返る。</x:v>
+      </x:c>
+      <x:c r="H59" t="str">
+        <x:v>取得客室IDが一致する。</x:v>
+      </x:c>
+      <x:c r="I59" t="str">
+        <x:v>API-010A / RULE-005</x:v>
+      </x:c>
+      <x:c r="J59" t="str">
+        <x:v>実施済</x:v>
+      </x:c>
+      <x:c r="K59" t="str">
+        <x:v>ReservationServiceLocalDbTest test_19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="15" hidden="0" customHeight="1">
+      <x:c r="A60" t="str">
+        <x:v>UT-044</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>ReservationService.syncTodayArrivals</x:v>
+      </x:c>
+      <x:c r="C60" t="str">
+        <x:v>当日到着を房態へ反映したい。</x:v>
+      </x:c>
+      <x:c r="D60" t="str">
+        <x:v>当日開始の booked 予約が reserved になること。</x:v>
+      </x:c>
+      <x:c r="E60" t="str">
+        <x:v>当日到着予約あり</x:v>
+      </x:c>
+      <x:c r="F60" t="str">
+        <x:v>syncTodayArrivals を実行</x:v>
+      </x:c>
+      <x:c r="G60" t="str">
+        <x:v>客室が reserved、清掃状態は維持。</x:v>
+      </x:c>
+      <x:c r="H60" t="str">
+        <x:v>DB状態が一致する。</x:v>
+      </x:c>
+      <x:c r="I60" t="str">
+        <x:v>BR-012 / LOGIC-009</x:v>
+      </x:c>
+      <x:c r="J60" t="str">
+        <x:v>実施済</x:v>
+      </x:c>
+      <x:c r="K60" t="str">
+        <x:v>ReservationServiceLocalDbTest test_20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="15" hidden="0" customHeight="1">
+      <x:c r="A61" t="str">
+        <x:v>UT-045</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>退室・清掃同期</x:v>
+      </x:c>
+      <x:c r="C61" t="str">
+        <x:v>同日後続予約の房態を保護したい。</x:v>
+      </x:c>
+      <x:c r="D61" t="str">
+        <x:v>退室・清掃更新後も後続予約があれば reserved を維持すること。</x:v>
+      </x:c>
+      <x:c r="E61" t="str">
+        <x:v>退室対象と同日後続予約あり</x:v>
+      </x:c>
+      <x:c r="F61" t="str">
+        <x:v>同期後に清掃済みへ更新</x:v>
+      </x:c>
+      <x:c r="G61" t="str">
+        <x:v>reserved を維持し清掃状態だけ更新。</x:v>
+      </x:c>
+      <x:c r="H61" t="str">
+        <x:v>DB状態が一致する。</x:v>
+      </x:c>
+      <x:c r="I61" t="str">
+        <x:v>REQ-009 / LOGIC-011</x:v>
+      </x:c>
+      <x:c r="J61" t="str">
+        <x:v>実施済</x:v>
+      </x:c>
+      <x:c r="K61" t="str">
+        <x:v>ReservationServiceLocalDbTest test_18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="36" customHeight="1">
+      <x:c r="A62" s="40" t="str">
+        <x:v>UT-CAL-001</x:v>
+      </x:c>
+      <x:c r="B62" s="40" t="str">
+        <x:v>RoomCalendarController</x:v>
+      </x:c>
+      <x:c r="C62" s="40" t="str">
+        <x:v>認証・CSRF</x:v>
+      </x:c>
+      <x:c r="D62" s="40" t="str">
+        <x:v>管理者認証あり</x:v>
+      </x:c>
+      <x:c r="E62" s="40" t="str">
+        <x:v>GETとPOSTを実行</x:v>
+      </x:c>
+      <x:c r="F62" s="40" t="str">
+        <x:v>未認証401、CSRFなし403、正常200/201</x:v>
+      </x:c>
+      <x:c r="G62" s="40" t="str">
+        <x:v>実施済</x:v>
+      </x:c>
+      <x:c r="H62" s="40" t="str">
+        <x:v>RoomCalendarControllerTest</x:v>
+      </x:c>
+      <x:c r="I62" s="40"/>
+      <x:c r="J62" s="40"/>
+      <x:c r="K62" s="40"/>
+    </x:row>
+    <x:row r="63" ht="36" customHeight="1">
+      <x:c r="A63" s="40" t="str">
+        <x:v>UT-CAL-002</x:v>
+      </x:c>
+      <x:c r="B63" s="40" t="str">
+        <x:v>RoomCalendarService</x:v>
+      </x:c>
+      <x:c r="C63" s="40" t="str">
+        <x:v>半開区間・競合</x:v>
+      </x:c>
+      <x:c r="D63" s="40" t="str">
+        <x:v>予約とブロックあり</x:v>
+      </x:c>
+      <x:c r="E63" s="40" t="str">
+        <x:v>境界日と重複期間を登録</x:v>
+      </x:c>
+      <x:c r="F63" s="40" t="str">
+        <x:v>同日入替可、重複409相当</x:v>
+      </x:c>
+      <x:c r="G63" s="40" t="str">
+        <x:v>実施済</x:v>
+      </x:c>
+      <x:c r="H63" s="40" t="str">
+        <x:v>RoomCalendarServiceLocalDbTest</x:v>
+      </x:c>
+      <x:c r="I63" s="40"/>
+      <x:c r="J63" s="40"/>
+      <x:c r="K63" s="40"/>
+    </x:row>
+    <x:row r="64" ht="36" customHeight="1">
+      <x:c r="A64" s="40" t="str">
+        <x:v>UT-CAL-003</x:v>
+      </x:c>
+      <x:c r="B64" s="40" t="str">
+        <x:v>在庫解除</x:v>
+      </x:c>
+      <x:c r="C64" s="40" t="str">
+        <x:v>全部・先頭・末尾・中間</x:v>
+      </x:c>
+      <x:c r="D64" s="40" t="str">
+        <x:v>有効ブロックあり</x:v>
+      </x:c>
+      <x:c r="E64" s="40" t="str">
+        <x:v>解除範囲を変更</x:v>
+      </x:c>
+      <x:c r="F64" s="40" t="str">
+        <x:v>取消または左右へ分割し監査記録</x:v>
+      </x:c>
+      <x:c r="G64" s="40" t="str">
+        <x:v>実施済</x:v>
+      </x:c>
+      <x:c r="H64" s="40" t="str">
+        <x:v>RoomCalendarServiceLocalDbTest</x:v>
+      </x:c>
+      <x:c r="I64" s="40"/>
+      <x:c r="J64" s="40"/>
+      <x:c r="K64" s="40"/>
+    </x:row>
+    <x:row r="65" ht="36" customHeight="1">
+      <x:c r="A65" s="40" t="str">
+        <x:v>UT-CAL-004</x:v>
+      </x:c>
+      <x:c r="B65" s="40" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="C65" s="40" t="str">
+        <x:v>GiST・trigger</x:v>
+      </x:c>
+      <x:c r="D65" s="40" t="str">
+        <x:v>実PostgreSQL</x:v>
+      </x:c>
+      <x:c r="E65" s="40" t="str">
+        <x:v>Flyway V5と競合書込を実行</x:v>
+      </x:c>
+      <x:c r="F65" s="40" t="str">
+        <x:v>DB制約で競合拒否</x:v>
+      </x:c>
+      <x:c r="G65" s="40" t="str">
+        <x:v>配備前確認</x:v>
+      </x:c>
+      <x:c r="H65" s="40" t="str">
+        <x:v>H2では検証不可</x:v>
+      </x:c>
+      <x:c r="I65" s="40"/>
+      <x:c r="J65" s="40"/>
+      <x:c r="K65" s="40"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3297,7 +3575,7 @@
         <x:v>何念童</x:v>
       </x:c>
       <x:c r="C3" s="27" t="str">
-        <x:v>2026-07-13</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="D3" s="27" t="str">
         <x:v>何念童</x:v>
@@ -3464,7 +3742,7 @@
         <x:v>何念童</x:v>
       </x:c>
       <x:c r="F11" s="30" t="str">
-        <x:v>JUnit5 106件、WebMvc、H2 DB連携、Scheduler、フロント build/lint、v1.9仕様書</x:v>
+        <x:v>JUnit5 123件、WebMvc、H2 DB連携、Scheduler、フロント build/lint、v1.10仕様書</x:v>
       </x:c>
       <x:c r="G11" s="30" t="str">
         <x:v>mvn test / npm lint / npm build / 全シート視覚確認</x:v>
@@ -3520,7 +3798,7 @@
         <x:v>何念童</x:v>
       </x:c>
       <x:c r="C3" s="27" t="str">
-        <x:v>2026-07-13</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="D3" s="27" t="str">
         <x:v>何念童</x:v>
@@ -3824,6 +4102,62 @@
       </x:c>
       <x:c r="D25" s="19" t="str">
         <x:v>src/test/java/com/example/minshuku/service/CheckoutSchedulerTest.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="36" customHeight="1">
+      <x:c r="A26" s="40" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B26" s="40" t="str">
+        <x:v>白馬樹海_管理端房態カレンダー仕様書.md</x:v>
+      </x:c>
+      <x:c r="C26" s="40" t="str">
+        <x:v>房態カレンダーの画面、API、DB、ロック、監査、受入条件。</x:v>
+      </x:c>
+      <x:c r="D26" s="40" t="str">
+        <x:v>docs/仕様書/白馬樹海_管理端房態カレンダー仕様書.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="36" customHeight="1">
+      <x:c r="A27" s="40" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B27" s="40" t="str">
+        <x:v>RoomCalendarService.java</x:v>
+      </x:c>
+      <x:c r="C27" s="40" t="str">
+        <x:v>月間投影と在庫・予約操作の業務ロジック。</x:v>
+      </x:c>
+      <x:c r="D27" s="40" t="str">
+        <x:v>src/main/java/com/example/minshuku/service/RoomCalendarService.java</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="36" customHeight="1">
+      <x:c r="A28" s="40" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B28" s="40" t="str">
+        <x:v>V5__room_inventory_calendar.sql</x:v>
+      </x:c>
+      <x:c r="C28" s="40" t="str">
+        <x:v>在庫ブロック、監査、排他制約、競合trigger。</x:v>
+      </x:c>
+      <x:c r="D28" s="40" t="str">
+        <x:v>src/main/resources/db/migration/V5__room_inventory_calendar.sql</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="36" customHeight="1">
+      <x:c r="A29" s="40" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B29" s="40" t="str">
+        <x:v>RoomCalendarControllerTest.java</x:v>
+      </x:c>
+      <x:c r="C29" s="40" t="str">
+        <x:v>認証、CSRF、正常、競合のWebMvcテスト。</x:v>
+      </x:c>
+      <x:c r="D29" s="40" t="str">
+        <x:v>src/test/java/com/example/minshuku/controller/RoomCalendarControllerTest.java</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3881,7 +4215,7 @@
         <x:v>何念童</x:v>
       </x:c>
       <x:c r="C3" s="39" t="str">
-        <x:v>2026-07-13</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="D3" s="39" t="str">
         <x:v>何念童</x:v>
@@ -3948,7 +4282,7 @@
         <x:v>期限到来チェックアウト</x:v>
       </x:c>
       <x:c r="D7" s="39" t="str">
-        <x:v>GET API は参照専用とし、CheckoutScheduler が既定で毎時0分に syncDueCheckouts を実行する。</x:v>
+        <x:v>GET API は参照専用とし、CheckoutScheduler が既定で毎分、syncDueCheckouts と syncTodayArrivals を実行する。</x:v>
       </x:c>
       <x:c r="E7" s="39" t="str">
         <x:v>GET 呼出しで更新されず、scheduler 単体テストと Service DBテストが成功すること。</x:v>
@@ -4115,6 +4449,46 @@
       </x:c>
       <x:c r="F15" s="19" t="str">
         <x:v>SecurityConfig.java / 配備設定</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="36" customHeight="1">
+      <x:c r="A16" s="40" t="str">
+        <x:v>OPS-CAL-001</x:v>
+      </x:c>
+      <x:c r="B16" s="40" t="str">
+        <x:v>運用</x:v>
+      </x:c>
+      <x:c r="C16" s="40" t="str">
+        <x:v>房態カレンダー</x:v>
+      </x:c>
+      <x:c r="D16" s="40" t="str">
+        <x:v>管理者画面は30秒更新と復帰時更新を行い、更新失敗時も直前表示を保持する。</x:v>
+      </x:c>
+      <x:c r="E16" s="40" t="str">
+        <x:v>可視状態と復帰時にAPI通信を確認する。</x:v>
+      </x:c>
+      <x:c r="F16" s="40" t="str">
+        <x:v>RoomCalendar.jsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="36" customHeight="1">
+      <x:c r="A17" s="40" t="str">
+        <x:v>OPS-CAL-002</x:v>
+      </x:c>
+      <x:c r="B17" s="40" t="str">
+        <x:v>DB</x:v>
+      </x:c>
+      <x:c r="C17" s="40" t="str">
+        <x:v>PostgreSQL V5</x:v>
+      </x:c>
+      <x:c r="D17" s="40" t="str">
+        <x:v>本番前にFlyway V5、GiST排他制約、相互競合triggerを実PostgreSQLで確認する。</x:v>
+      </x:c>
+      <x:c r="E17" s="40" t="str">
+        <x:v>mvn verifyに加え実DB統合試験を実施する。</x:v>
+      </x:c>
+      <x:c r="F17" s="40" t="str">
+        <x:v>V5__room_inventory_calendar.sql</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4169,7 +4543,7 @@
         <x:v>何念童</x:v>
       </x:c>
       <x:c r="C3" s="27" t="str">
-        <x:v>2026-07-13</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="D3" s="27" t="str">
         <x:v>何念童</x:v>
@@ -4364,6 +4738,36 @@
         <x:v>何念童</x:v>
       </x:c>
       <x:c r="E16" s="19"/>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" t="str">
+        <x:v>1.10</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>2026-09-02</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>宿泊数自動計算、日程・人数別の空室候補、到着日房態同期、同日後続予約を保護する清掃・退室同期を実装とテストへ反映</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>何念童</x:v>
+      </x:c>
+      <x:c r="E17"/>
+    </x:row>
+    <x:row r="18" ht="36" customHeight="1">
+      <x:c r="A18" s="40" t="str">
+        <x:v>1.11</x:v>
+      </x:c>
+      <x:c r="B18" s="40" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="C18" s="40" t="str">
+        <x:v>管理端房態カレンダー、在庫ブロック、半開区間、競合制御、監査、30秒更新、関連テストを反映</x:v>
+      </x:c>
+      <x:c r="D18" s="40" t="str">
+        <x:v>何念童</x:v>
+      </x:c>
+      <x:c r="E18" s="40"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4414,7 +4818,7 @@
         <x:v>何念童</x:v>
       </x:c>
       <x:c r="C3" s="27" t="str">
-        <x:v>2026-07-13</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="D3" s="27" t="str">
         <x:v>何念童</x:v>
@@ -4521,7 +4925,7 @@
         <x:v>民宿運用では、予約、客室状態、清掃状態、期間別料金を一元管理する必要がある。</x:v>
       </x:c>
       <x:c r="D11" s="30" t="str">
-        <x:v>業務上の必要性を確認する。</x:v>
+        <x:v>予約日程・人数と実房態の整合性を確認する。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -4723,7 +5127,7 @@
         <x:v>チェックアウト同期</x:v>
       </x:c>
       <x:c r="D26" s="19" t="str">
-        <x:v>@EnableScheduling と CheckoutScheduler により毎時0分（Asia/Tokyo）に期限到来予約を同期し、GET API は更新を行わない。</x:v>
+        <x:v>@EnableScheduling と CheckoutScheduler により毎分（Asia/Tokyo）に期限到来チェックアウトと当日到着予約を同期し、GET API は更新を行わない。</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -4738,6 +5142,34 @@
       </x:c>
       <x:c r="D27" s="19" t="str">
         <x:v>予約中・取消済み・チェックアウト済みを独立した5件ページで返し、各 PageResponse に totalCount を含める。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="36" customHeight="1">
+      <x:c r="A28" s="40" t="str">
+        <x:v>BASE-013</x:v>
+      </x:c>
+      <x:c r="B28" s="40" t="str">
+        <x:v>在庫管理</x:v>
+      </x:c>
+      <x:c r="C28" s="40" t="str">
+        <x:v>管理端房態カレンダー</x:v>
+      </x:c>
+      <x:c r="D28" s="40" t="str">
+        <x:v>自然月 Tape Chart で予約、販売停止、メンテナンスを客室別に一元表示する。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="36" customHeight="1">
+      <x:c r="A29" s="40" t="str">
+        <x:v>BASE-014</x:v>
+      </x:c>
+      <x:c r="B29" s="40" t="str">
+        <x:v>期間規則</x:v>
+      </x:c>
+      <x:c r="C29" s="40" t="str">
+        <x:v>半開区間</x:v>
+      </x:c>
+      <x:c r="D29" s="40" t="str">
+        <x:v>予約・在庫ブロックは [開始日, 退房日／販売再開日) で判定し、終了日は占有しない。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4794,7 +5226,7 @@
         <x:v>何念童</x:v>
       </x:c>
       <x:c r="C3" s="27" t="str">
-        <x:v>2026-07-13</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="D3" s="27" t="str">
         <x:v>何念童</x:v>
@@ -4857,7 +5289,7 @@
         <x:v>予約登録</x:v>
       </x:c>
       <x:c r="D7" s="30" t="str">
-        <x:v>空室かつ清掃済みの客室に対して、宿泊者・日程・人数・同行者を登録できる。</x:v>
+        <x:v>日程・人数に合い、他予約と重複しない有効客室に対して、宿泊者・同行者を登録できる。</x:v>
       </x:c>
       <x:c r="E7" s="30" t="str">
         <x:v>高</x:v>
@@ -5077,7 +5509,7 @@
         <x:v>料金重複防止</x:v>
       </x:c>
       <x:c r="D18" s="30" t="str">
-        <x:v>同一客室で期間が重なる料金ルールを拒否する。</x:v>
+        <x:v>宿泊終了日を迎えた予約をチェックアウト済みにし、当日到着予約を予約済み房態へ同期する。</x:v>
       </x:c>
       <x:c r="E18" s="30" t="str">
         <x:v>高</x:v>
@@ -5377,7 +5809,7 @@
         <x:v>清掃管理</x:v>
       </x:c>
       <x:c r="D33" s="30" t="str">
-        <x:v>チェックアウト後の清掃状態を管理できること。</x:v>
+        <x:v>チェックアウト後の清掃状態を管理し、同日に他の予約がある場合はその予約の宿泊状態を維持できること。</x:v>
       </x:c>
       <x:c r="E33" s="30" t="str">
         <x:v>checked_out 予約の客室を needs_cleaning / cleaned に更新できる。</x:v>
@@ -5417,7 +5849,7 @@
         <x:v>ダッシュボード</x:v>
       </x:c>
       <x:c r="D35" s="30" t="str">
-        <x:v>現在の客室・予約状況を参照できること。</x:v>
+        <x:v>CheckoutScheduler が毎分、期限到来チェックアウトと当日到着を同期した永続化済み状態を GET API が読取専用で返す。</x:v>
       </x:c>
       <x:c r="E35" s="30" t="str">
         <x:v>CheckoutScheduler が定期同期した永続化済み状態を GET API が読取専用で返す。</x:v>
@@ -5577,7 +6009,7 @@
         <x:v>客室検証</x:v>
       </x:c>
       <x:c r="D43" s="30" t="str">
-        <x:v>active=true、occupancy_status=vacant、cleaning_status=cleaned、人数 &lt;= 定員</x:v>
+        <x:v>active=true、人数&lt;=定員、対象期間に有効予約との重複なし。当日入室は vacant / cleaned も満たす。</x:v>
       </x:c>
       <x:c r="E43" s="30" t="str">
         <x:v>予約対象として確定</x:v>
@@ -5797,13 +6229,53 @@
         <x:v>CheckoutScheduler 実行時</x:v>
       </x:c>
       <x:c r="D54" s="19" t="str">
-        <x:v>booked かつ check_out_date &lt;= DB CURRENT_DATE</x:v>
+        <x:v>booked かつ check_out_date &lt;= DB CURRENT_DATE、または booked かつ check_in_date = DB CURRENT_DATE</x:v>
       </x:c>
       <x:c r="E54" s="19" t="str">
-        <x:v>予約を checked_out、客室を vacant / needs_cleaning に同期</x:v>
+        <x:v>退室は checked_out、当日到着は reserved。清掃更新時も他予約に合わせて occupied / reserved / vacant を再計算</x:v>
       </x:c>
       <x:c r="F54" s="19" t="str">
         <x:v>GET /dashboard・/reservations は状態更新しない</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="36" customHeight="1">
+      <x:c r="A55" s="40" t="str">
+        <x:v>CAL-BR-001</x:v>
+      </x:c>
+      <x:c r="B55" s="40" t="str">
+        <x:v>房態</x:v>
+      </x:c>
+      <x:c r="C55" s="40" t="str">
+        <x:v>月間房態表示</x:v>
+      </x:c>
+      <x:c r="D55" s="40" t="str">
+        <x:v>管理者が自然月単位で全客室の予約・販売停止・メンテナンスを確認できる。</x:v>
+      </x:c>
+      <x:c r="E55" s="40" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="F55" s="40" t="str">
+        <x:v>RoomCalendar</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="36" customHeight="1">
+      <x:c r="A56" s="40" t="str">
+        <x:v>CAL-RULE-001</x:v>
+      </x:c>
+      <x:c r="B56" s="40" t="str">
+        <x:v>競合制御</x:v>
+      </x:c>
+      <x:c r="C56" s="40" t="str">
+        <x:v>在庫更新</x:v>
+      </x:c>
+      <x:c r="D56" s="40" t="str">
+        <x:v>客室行をロック後、予約と有効ブロックの重複を再検証する。</x:v>
+      </x:c>
+      <x:c r="E56" s="40" t="str">
+        <x:v>競合なしなら同一トランザクションで保存</x:v>
+      </x:c>
+      <x:c r="F56" s="40" t="str">
+        <x:v>競合時は HTTP 409</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5869,7 +6341,7 @@
         <x:v>何念童</x:v>
       </x:c>
       <x:c r="C3" s="27" t="str">
-        <x:v>2026-07-13</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="D3" s="27" t="str">
         <x:v>何念童</x:v>
@@ -6008,7 +6480,7 @@
         <x:v>予約登録</x:v>
       </x:c>
       <x:c r="D9" s="30" t="str">
-        <x:v>入力検証、客室ロック、重複確認、料金計算、同行者保存を行う。</x:v>
+        <x:v>宿泊数を日付差で算出し、日程・人数で空室候補を取得後、入力検証・客室ロック・重複確認・料金計算・同行者保存を行う。</x:v>
       </x:c>
       <x:c r="E9" s="30" t="str">
         <x:v>ReservationCreateRequest</x:v>
@@ -6153,7 +6625,7 @@
         <x:v>清掃状態更新</x:v>
       </x:c>
       <x:c r="D14" s="30" t="str">
-        <x:v>チェックアウト後の客室清掃状態を更新する。</x:v>
+        <x:v>チェックアウト後の清掃状態を更新し、同日後続予約または滞在中予約の宿泊状態を維持する。</x:v>
       </x:c>
       <x:c r="E14" s="30" t="str">
         <x:v>CleaningRequest</x:v>
@@ -6414,7 +6886,7 @@
         <x:v>定期チェックアウト同期</x:v>
       </x:c>
       <x:c r="D23" s="19" t="str">
-        <x:v>毎時0分に期限到来予約を同期し、参照APIから更新処理を分離する。</x:v>
+        <x:v>毎分、期限到来チェックアウトと当日到着予約を同期し、参照APIから更新処理を分離する。</x:v>
       </x:c>
       <x:c r="E23" s="19" t="str">
         <x:v>cron / timezone</x:v>
@@ -6733,10 +7205,10 @@
         <x:v>ApiController</x:v>
       </x:c>
       <x:c r="D34" s="30" t="str">
-        <x:v>deleteCancelledReservation</x:v>
+        <x:v>日程・人数を受け取り、期間重複・定員・当日房態を判定して予約可能客室を返す。</x:v>
       </x:c>
       <x:c r="E34" s="30" t="str">
-        <x:v>取消済み予約削除 API を受け取り、Service の deleteCancelled へ委譲する。</x:v>
+        <x:v>GET /api/reservations/available-rooms</x:v>
       </x:c>
       <x:c r="F34" s="30" t="str">
         <x:v>POST /api/reservations/{id}/delete</x:v>
@@ -6907,7 +7379,7 @@
         <x:v>ReservationService</x:v>
       </x:c>
       <x:c r="D40" s="30" t="str">
-        <x:v>syncDueCheckouts</x:v>
+        <x:v>期限到来予約を checked_out にし、同日他予約を確認して客室を occupied / reserved / vacant と needs_cleaning に同期する。</x:v>
       </x:c>
       <x:c r="E40" s="30" t="str">
         <x:v>booked かつ check_out_date &lt;= CURRENT_DATE の予約を checked_out にし、客室を vacant / needs_cleaning にする。</x:v>
@@ -6965,7 +7437,7 @@
         <x:v>ReservationService</x:v>
       </x:c>
       <x:c r="D42" s="30" t="str">
-        <x:v>updateCheckoutCleaningStatus</x:v>
+        <x:v>checked_out 予約の清掃状態を更新し、同日他予約の状態を優先して客室の宿泊状態を再計算する。</x:v>
       </x:c>
       <x:c r="E42" s="30" t="str">
         <x:v>予約を取得し、checked_out 予約だけ清掃状態許可値を検証して客室を vacant のまま更新する。</x:v>
@@ -7139,7 +7611,7 @@
         <x:v>RoomMapper.xml</x:v>
       </x:c>
       <x:c r="D48" s="30" t="str">
-        <x:v>findBookable</x:v>
+        <x:v>findAvailableForStay で active、定員、期間重複、当日 vacant / cleaned を判定して候補を取得する。</x:v>
       </x:c>
       <x:c r="E48" s="30" t="str">
         <x:v>active=true、vacant、cleaned の客室を予約フォーム候補として取得する。</x:v>
@@ -7226,7 +7698,7 @@
         <x:v>CheckoutScheduler</x:v>
       </x:c>
       <x:c r="D51" s="19" t="str">
-        <x:v>syncDueCheckouts</x:v>
+        <x:v>設定可能な cron / timezone で syncDueCheckouts と syncTodayArrivals を順に実行する。</x:v>
       </x:c>
       <x:c r="E51" s="19" t="str">
         <x:v>設定可能な cron / timezone で ReservationService.syncDueCheckouts を委譲実行する。</x:v>
@@ -7241,7 +7713,7 @@
         <x:v>Service側</x:v>
       </x:c>
       <x:c r="I51" s="19" t="str">
-        <x:v>既定: 0 0 * * * * / Asia/Tokyo</x:v>
+        <x:v>既定: 0 * * * * * / Asia/Tokyo</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
@@ -7757,6 +8229,118 @@
         <x:v>ReservationService へ委譲</x:v>
       </x:c>
       <x:c r="I71" s="19"/>
+    </x:row>
+    <x:row r="72" ht="36" customHeight="1">
+      <x:c r="A72" s="40" t="str">
+        <x:v>F-CAL-001</x:v>
+      </x:c>
+      <x:c r="B72" s="40" t="str">
+        <x:v>房態</x:v>
+      </x:c>
+      <x:c r="C72" s="40" t="str">
+        <x:v>自然月カレンダー</x:v>
+      </x:c>
+      <x:c r="D72" s="40" t="str">
+        <x:v>客室行×日付列の Tape Chart を表示し、予約と在庫ブロックを帯で示す。</x:v>
+      </x:c>
+      <x:c r="E72" s="40" t="str">
+        <x:v>month</x:v>
+      </x:c>
+      <x:c r="F72" s="40" t="str">
+        <x:v>CalendarView</x:v>
+      </x:c>
+      <x:c r="G72" s="40" t="str">
+        <x:v>管理者</x:v>
+      </x:c>
+      <x:c r="H72" s="40" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I72" s="40" t="str">
+        <x:v>RoomCalendarController / RoomCalendarService</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="36" customHeight="1">
+      <x:c r="A73" s="40" t="str">
+        <x:v>F-CAL-002</x:v>
+      </x:c>
+      <x:c r="B73" s="40" t="str">
+        <x:v>在庫</x:v>
+      </x:c>
+      <x:c r="C73" s="40" t="str">
+        <x:v>販売停止・メンテナンス</x:v>
+      </x:c>
+      <x:c r="D73" s="40" t="str">
+        <x:v>空き期間からブロックを作成・更新・全部／一部解除する。</x:v>
+      </x:c>
+      <x:c r="E73" s="40" t="str">
+        <x:v>roomId / blockType / [start,end)</x:v>
+      </x:c>
+      <x:c r="F73" s="40" t="str">
+        <x:v>BlockView</x:v>
+      </x:c>
+      <x:c r="G73" s="40" t="str">
+        <x:v>管理者</x:v>
+      </x:c>
+      <x:c r="H73" s="40" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I73" s="40" t="str">
+        <x:v>RoomCalendarService</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="36" customHeight="1">
+      <x:c r="A74" s="40" t="str">
+        <x:v>JAVA-CAL-001</x:v>
+      </x:c>
+      <x:c r="B74" s="40" t="str">
+        <x:v>service</x:v>
+      </x:c>
+      <x:c r="C74" s="40" t="str">
+        <x:v>RoomCalendarService</x:v>
+      </x:c>
+      <x:c r="D74" s="40" t="str">
+        <x:v>月間投影、競合判定、ロック、分割解除、監査記録、予約操作を担当する。</x:v>
+      </x:c>
+      <x:c r="E74" s="40" t="str">
+        <x:v>calendar / createBlock / releaseBlock</x:v>
+      </x:c>
+      <x:c r="F74" s="40" t="str">
+        <x:v>RoomInventoryMapper</x:v>
+      </x:c>
+      <x:c r="G74" s="40" t="str">
+        <x:v>業務ロジック</x:v>
+      </x:c>
+      <x:c r="H74" s="40" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I74" s="40"/>
+    </x:row>
+    <x:row r="75" ht="36" customHeight="1">
+      <x:c r="A75" s="40" t="str">
+        <x:v>JAVA-CAL-002</x:v>
+      </x:c>
+      <x:c r="B75" s="40" t="str">
+        <x:v>mapper</x:v>
+      </x:c>
+      <x:c r="C75" s="40" t="str">
+        <x:v>RoomInventoryMapper</x:v>
+      </x:c>
+      <x:c r="D75" s="40" t="str">
+        <x:v>在庫ブロックと追記型監査イベントを永続化する。</x:v>
+      </x:c>
+      <x:c r="E75" s="40" t="str">
+        <x:v>findEffective / insert / cancel / insertEvent</x:v>
+      </x:c>
+      <x:c r="F75" s="40" t="str">
+        <x:v>RoomInventoryMapper.xml</x:v>
+      </x:c>
+      <x:c r="G75" s="40" t="str">
+        <x:v>DAO</x:v>
+      </x:c>
+      <x:c r="H75" s="40" t="str">
+        <x:v>高</x:v>
+      </x:c>
+      <x:c r="I75" s="40"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -7807,7 +8391,7 @@
         <x:v>何念童</x:v>
       </x:c>
       <x:c r="C3" s="27" t="str">
-        <x:v>2026-07-13</x:v>
+        <x:v>2026-09-02</x:v>
       </x:c>
       <x:c r="D3" s="27" t="str">
         <x:v>何念童</x:v>
@@ -11368,7 +11952,7 @@
         <x:v>何念童</x:v>
       </x:c>
       <x:c r="C3" s="27" t="str">
-        <x:v>2026-07-13</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="D3" s="27" t="str">
         <x:v>何念童</x:v>
@@ -11640,6 +12224,52 @@
       </x:c>
       <x:c r="G16" s="30" t="str">
         <x:v>料金ルールは予約金額計算の根拠として使用する。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="36" customHeight="1">
+      <x:c r="A17" s="40" t="str">
+        <x:v>S-CAL-001</x:v>
+      </x:c>
+      <x:c r="B17" s="40" t="str">
+        <x:v>房態カレンダー</x:v>
+      </x:c>
+      <x:c r="C17" s="40" t="str">
+        <x:v>管理者</x:v>
+      </x:c>
+      <x:c r="D17" s="40" t="str">
+        <x:v>自然月の全客室を横軸日付の Tape Chart で確認・操作する。</x:v>
+      </x:c>
+      <x:c r="E17" s="40" t="str">
+        <x:v>月移動、予約帯、販売停止、メンテナンス、詳細モーダル</x:v>
+      </x:c>
+      <x:c r="F17" s="40" t="str">
+        <x:v>共通ナビ</x:v>
+      </x:c>
+      <x:c r="G17" s="40" t="str">
+        <x:v>同画面</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="36" customHeight="1">
+      <x:c r="A18" s="40" t="str">
+        <x:v>SCR-CAL-001</x:v>
+      </x:c>
+      <x:c r="B18" s="40" t="str">
+        <x:v>/jukai-internal/calendar</x:v>
+      </x:c>
+      <x:c r="C18" s="40" t="str">
+        <x:v>DashboardController</x:v>
+      </x:c>
+      <x:c r="D18" s="40" t="str">
+        <x:v>GET /api/room-calendar</x:v>
+      </x:c>
+      <x:c r="E18" s="40" t="str">
+        <x:v>rooms / stays / blocks / today</x:v>
+      </x:c>
+      <x:c r="F18" s="40" t="str">
+        <x:v>空き期間選択、予約・ブロック操作</x:v>
+      </x:c>
+      <x:c r="G18" s="40" t="str">
+        <x:v>30秒更新。詳細は選択時に取得。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -11699,7 +12329,7 @@
         <x:v>何念童</x:v>
       </x:c>
       <x:c r="C3" s="27" t="str">
-        <x:v>2026-07-13</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="D3" s="27" t="str">
         <x:v>何念童</x:v>
@@ -11930,24 +12560,24 @@
         <x:v>論理削除フラグ。</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="24" hidden="0" customHeight="1">
-      <x:c r="A16" s="30" t="str">
+    <x:row r="16" ht="36" hidden="0" customHeight="1">
+      <x:c r="A16" s="41" t="str">
         <x:v>reservations</x:v>
       </x:c>
-      <x:c r="B16" s="30" t="str">
+      <x:c r="B16" s="41" t="str">
         <x:v>id</x:v>
       </x:c>
-      <x:c r="C16" s="30" t="str">
+      <x:c r="C16" s="41" t="str">
         <x:v>INTEGER GENERATED BY DEFAULT AS IDENTITY</x:v>
       </x:c>
-      <x:c r="D16" s="30" t="str">
+      <x:c r="D16" s="41" t="str">
         <x:v>YES</x:v>
       </x:c>
-      <x:c r="E16" s="30"/>
-      <x:c r="F16" s="30" t="str">
+      <x:c r="E16" s="41"/>
+      <x:c r="F16" s="41" t="str">
         <x:v>NO</x:v>
       </x:c>
-      <x:c r="G16" s="30" t="str">
+      <x:c r="G16" s="41" t="str">
         <x:v>予約ID。</x:v>
       </x:c>
     </x:row>
@@ -13346,6 +13976,166 @@
       </x:c>
       <x:c r="G83" s="19" t="str">
         <x:v>本番Flywayとは別管理</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="36" customHeight="1">
+      <x:c r="A84" s="40" t="str">
+        <x:v>room_inventory_blocks</x:v>
+      </x:c>
+      <x:c r="B84" s="40" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="C84" s="40" t="str">
+        <x:v>BIGINT GENERATED BY DEFAULT AS IDENTITY</x:v>
+      </x:c>
+      <x:c r="D84" s="40" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="E84" s="40"/>
+      <x:c r="F84" s="40" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G84" s="40" t="str">
+        <x:v>在庫ブロックID。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="36" customHeight="1">
+      <x:c r="A85" s="40" t="str">
+        <x:v>room_inventory_blocks</x:v>
+      </x:c>
+      <x:c r="B85" s="40" t="str">
+        <x:v>room_id</x:v>
+      </x:c>
+      <x:c r="C85" s="40" t="str">
+        <x:v>BIGINT</x:v>
+      </x:c>
+      <x:c r="D85" s="40"/>
+      <x:c r="E85" s="40" t="str">
+        <x:v>rooms.id</x:v>
+      </x:c>
+      <x:c r="F85" s="40" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G85" s="40" t="str">
+        <x:v>対象客室。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="36" customHeight="1">
+      <x:c r="A86" s="40" t="str">
+        <x:v>room_inventory_blocks</x:v>
+      </x:c>
+      <x:c r="B86" s="40" t="str">
+        <x:v>block_type</x:v>
+      </x:c>
+      <x:c r="C86" s="40" t="str">
+        <x:v>VARCHAR(20)</x:v>
+      </x:c>
+      <x:c r="D86" s="40"/>
+      <x:c r="E86" s="40"/>
+      <x:c r="F86" s="40" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G86" s="40" t="str">
+        <x:v>stop_sale / maintenance。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="36" customHeight="1">
+      <x:c r="A87" s="40" t="str">
+        <x:v>room_inventory_blocks</x:v>
+      </x:c>
+      <x:c r="B87" s="40" t="str">
+        <x:v>start_date / end_date</x:v>
+      </x:c>
+      <x:c r="C87" s="40" t="str">
+        <x:v>DATE</x:v>
+      </x:c>
+      <x:c r="D87" s="40"/>
+      <x:c r="E87" s="40"/>
+      <x:c r="F87" s="40" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G87" s="40" t="str">
+        <x:v>DB上の半開区間 [start,end)。APIではendDateExclusive。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="36" customHeight="1">
+      <x:c r="A88" s="40" t="str">
+        <x:v>room_inventory_blocks</x:v>
+      </x:c>
+      <x:c r="B88" s="40" t="str">
+        <x:v>record_status / version</x:v>
+      </x:c>
+      <x:c r="C88" s="40" t="str">
+        <x:v>VARCHAR / INTEGER</x:v>
+      </x:c>
+      <x:c r="D88" s="40"/>
+      <x:c r="E88" s="40"/>
+      <x:c r="F88" s="40" t="str">
+        <x:v>NO</x:v>
+      </x:c>
+      <x:c r="G88" s="40" t="str">
+        <x:v>有効状態と楽観ロック版。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="36" customHeight="1">
+      <x:c r="A89" s="40" t="str">
+        <x:v>room_inventory_block_events</x:v>
+      </x:c>
+      <x:c r="B89" s="40" t="str">
+        <x:v>before_* / after_*</x:v>
+      </x:c>
+      <x:c r="C89" s="40" t="str">
+        <x:v>VARCHAR / DATE</x:v>
+      </x:c>
+      <x:c r="D89" s="40"/>
+      <x:c r="E89" s="40"/>
+      <x:c r="F89" s="40" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="G89" s="40" t="str">
+        <x:v>種別・期間・理由・状態の変更前後を列別に追記監査。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="36" customHeight="1">
+      <x:c r="A90" s="40" t="str">
+        <x:v>reservations</x:v>
+      </x:c>
+      <x:c r="B90" s="40" t="str">
+        <x:v>cancellation_reason / cancelled_by / cancelled_at</x:v>
+      </x:c>
+      <x:c r="C90" s="40" t="str">
+        <x:v>VARCHAR / VARCHAR / TIMESTAMPTZ</x:v>
+      </x:c>
+      <x:c r="D90" s="40"/>
+      <x:c r="E90" s="40"/>
+      <x:c r="F90" s="40" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+      <x:c r="G90" s="40" t="str">
+        <x:v>取消理由・操作者・時刻。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="36" customHeight="1">
+      <x:c r="A91" s="40" t="str">
+        <x:v>MIG-005</x:v>
+      </x:c>
+      <x:c r="B91" s="40" t="str">
+        <x:v>Flyway</x:v>
+      </x:c>
+      <x:c r="C91" s="40" t="str">
+        <x:v>V5__room_inventory_calendar.sql</x:v>
+      </x:c>
+      <x:c r="D91" s="40" t="str">
+        <x:v>在庫テーブル、監査、GiST排他制約、予約との相互競合trigger</x:v>
+      </x:c>
+      <x:c r="E91" s="40" t="str">
+        <x:v>アプリ起動時</x:v>
+      </x:c>
+      <x:c r="F91" s="40" t="str">
+        <x:v>PostgreSQL</x:v>
+      </x:c>
+      <x:c r="G91" s="40" t="str">
+        <x:v>H2ではService競合テストを実施</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -13408,7 +14198,7 @@
         <x:v>何念童</x:v>
       </x:c>
       <x:c r="C3" s="27" t="str">
-        <x:v>2026-07-13</x:v>
+        <x:v>2026-09-30</x:v>
       </x:c>
       <x:c r="D3" s="27" t="str">
         <x:v>何念童</x:v>
@@ -13957,7 +14747,7 @@
         <x:v>清掃状態更新</x:v>
       </x:c>
       <x:c r="F25" s="30" t="str">
-        <x:v>CleaningRequest</x:v>
+        <x:v>CleaningRequest（同日他予約の宿泊状態を保護）</x:v>
       </x:c>
       <x:c r="G25" s="30" t="str">
         <x:v>MessageResponse</x:v>
@@ -13993,14 +14783,30 @@
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
-      <x:c r="A27" s="19"/>
-      <x:c r="B27" s="19"/>
-      <x:c r="C27" s="19"/>
-      <x:c r="D27" s="19"/>
-      <x:c r="E27" s="19"/>
-      <x:c r="F27" s="19"/>
-      <x:c r="G27" s="19"/>
-      <x:c r="H27" s="19"/>
+      <x:c r="A27" s="19" t="str">
+        <x:v>API-010A</x:v>
+      </x:c>
+      <x:c r="B27" s="19" t="str">
+        <x:v>Reservation</x:v>
+      </x:c>
+      <x:c r="C27" s="19" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="D27" s="19" t="str">
+        <x:v>/api/reservations/available-rooms</x:v>
+      </x:c>
+      <x:c r="E27" s="19" t="str">
+        <x:v>宿泊日程・人数に合う予約可能客室を取得</x:v>
+      </x:c>
+      <x:c r="F27" s="19" t="str">
+        <x:v>checkInDate / checkOutDate / guestCount</x:v>
+      </x:c>
+      <x:c r="G27" s="19" t="str">
+        <x:v>List&lt;Room&gt;</x:v>
+      </x:c>
+      <x:c r="H27" s="19" t="str">
+        <x:v>アプリ内認証なし（社内NW/Proxy前提）</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="26" t="str">
@@ -14718,6 +15524,214 @@
       </x:c>
       <x:c r="H56" s="30"/>
     </x:row>
+    <x:row r="57" ht="36" customHeight="1">
+      <x:c r="A57" s="40" t="str">
+        <x:v>API-CAL-001</x:v>
+      </x:c>
+      <x:c r="B57" s="40" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="C57" s="40" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="D57" s="40" t="str">
+        <x:v>/api/room-calendar?month=YYYY-MM</x:v>
+      </x:c>
+      <x:c r="E57" s="40" t="str">
+        <x:v>自然月の客室・予約・ブロック取得</x:v>
+      </x:c>
+      <x:c r="F57" s="40" t="str">
+        <x:v>month</x:v>
+      </x:c>
+      <x:c r="G57" s="40" t="str">
+        <x:v>CalendarView</x:v>
+      </x:c>
+      <x:c r="H57" s="40" t="str">
+        <x:v>管理者</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="36" customHeight="1">
+      <x:c r="A58" s="40" t="str">
+        <x:v>API-CAL-002</x:v>
+      </x:c>
+      <x:c r="B58" s="40" t="str">
+        <x:v>Calendar</x:v>
+      </x:c>
+      <x:c r="C58" s="40" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="D58" s="40" t="str">
+        <x:v>/api/room-calendar/reservations/{id}</x:v>
+      </x:c>
+      <x:c r="E58" s="40" t="str">
+        <x:v>予約詳細と許可操作取得</x:v>
+      </x:c>
+      <x:c r="F58" s="40" t="str">
+        <x:v>id</x:v>
+      </x:c>
+      <x:c r="G58" s="40" t="str">
+        <x:v>ReservationDetail</x:v>
+      </x:c>
+      <x:c r="H58" s="40" t="str">
+        <x:v>管理者</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="36" customHeight="1">
+      <x:c r="A59" s="40" t="str">
+        <x:v>API-CAL-003</x:v>
+      </x:c>
+      <x:c r="B59" s="40" t="str">
+        <x:v>Inventory</x:v>
+      </x:c>
+      <x:c r="C59" s="40" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="D59" s="40" t="str">
+        <x:v>/api/room-calendar/blocks</x:v>
+      </x:c>
+      <x:c r="E59" s="40" t="str">
+        <x:v>在庫ブロック作成</x:v>
+      </x:c>
+      <x:c r="F59" s="40" t="str">
+        <x:v>blockType / roomId / [start,end)</x:v>
+      </x:c>
+      <x:c r="G59" s="40" t="str">
+        <x:v>BlockView</x:v>
+      </x:c>
+      <x:c r="H59" s="40" t="str">
+        <x:v>管理者</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="36" customHeight="1">
+      <x:c r="A60" s="40" t="str">
+        <x:v>API-CAL-004</x:v>
+      </x:c>
+      <x:c r="B60" s="40" t="str">
+        <x:v>Inventory</x:v>
+      </x:c>
+      <x:c r="C60" s="40" t="str">
+        <x:v>PUT</x:v>
+      </x:c>
+      <x:c r="D60" s="40" t="str">
+        <x:v>/api/room-calendar/blocks/{id}</x:v>
+      </x:c>
+      <x:c r="E60" s="40" t="str">
+        <x:v>在庫ブロック更新</x:v>
+      </x:c>
+      <x:c r="F60" s="40" t="str">
+        <x:v>version / period / reason</x:v>
+      </x:c>
+      <x:c r="G60" s="40" t="str">
+        <x:v>BlockView</x:v>
+      </x:c>
+      <x:c r="H60" s="40" t="str">
+        <x:v>管理者</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="36" customHeight="1">
+      <x:c r="A61" s="40" t="str">
+        <x:v>API-CAL-005</x:v>
+      </x:c>
+      <x:c r="B61" s="40" t="str">
+        <x:v>Inventory</x:v>
+      </x:c>
+      <x:c r="C61" s="40" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="D61" s="40" t="str">
+        <x:v>/api/room-calendar/blocks/{id}/release</x:v>
+      </x:c>
+      <x:c r="E61" s="40" t="str">
+        <x:v>全部／一部解除</x:v>
+      </x:c>
+      <x:c r="F61" s="40" t="str">
+        <x:v>[releaseStart,releaseEnd)</x:v>
+      </x:c>
+      <x:c r="G61" s="40" t="str">
+        <x:v>ReleaseResult</x:v>
+      </x:c>
+      <x:c r="H61" s="40" t="str">
+        <x:v>管理者</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="36" customHeight="1">
+      <x:c r="A62" s="40" t="str">
+        <x:v>API-CAL-006</x:v>
+      </x:c>
+      <x:c r="B62" s="40" t="str">
+        <x:v>Booking</x:v>
+      </x:c>
+      <x:c r="C62" s="40" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="D62" s="40" t="str">
+        <x:v>/api/booking-requests/{id}/cancel</x:v>
+      </x:c>
+      <x:c r="E62" s="40" t="str">
+        <x:v>公開予約をグループ単位で取消</x:v>
+      </x:c>
+      <x:c r="F62" s="40" t="str">
+        <x:v>reason</x:v>
+      </x:c>
+      <x:c r="G62" s="40" t="str">
+        <x:v>MessageResponse</x:v>
+      </x:c>
+      <x:c r="H62" s="40" t="str">
+        <x:v>管理者</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="36" customHeight="1">
+      <x:c r="A63" s="40" t="str">
+        <x:v>API-CAL-007</x:v>
+      </x:c>
+      <x:c r="B63" s="40" t="str">
+        <x:v>Room</x:v>
+      </x:c>
+      <x:c r="C63" s="40" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="D63" s="40" t="str">
+        <x:v>/api/rooms/{id}/cleaning-status</x:v>
+      </x:c>
+      <x:c r="E63" s="40" t="str">
+        <x:v>清掃状態更新</x:v>
+      </x:c>
+      <x:c r="F63" s="40" t="str">
+        <x:v>cleaningStatus</x:v>
+      </x:c>
+      <x:c r="G63" s="40" t="str">
+        <x:v>MessageResponse</x:v>
+      </x:c>
+      <x:c r="H63" s="40" t="str">
+        <x:v>管理者</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="36" customHeight="1">
+      <x:c r="A64" s="40" t="str">
+        <x:v>API-CAL-008</x:v>
+      </x:c>
+      <x:c r="B64" s="40" t="str">
+        <x:v>Reservation</x:v>
+      </x:c>
+      <x:c r="C64" s="40" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="D64" s="40" t="str">
+        <x:v>/api/reservations/{id}/cancel</x:v>
+      </x:c>
+      <x:c r="E64" s="40" t="str">
+        <x:v>直接予約取消と理由保存</x:v>
+      </x:c>
+      <x:c r="F64" s="40" t="str">
+        <x:v>reason（任意）</x:v>
+      </x:c>
+      <x:c r="G64" s="40" t="str">
+        <x:v>MessageResponse</x:v>
+      </x:c>
+      <x:c r="H64" s="40" t="str">
+        <x:v>管理者</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>

</xml_diff>